<commit_message>
test(calculators): got feed purchase tests to pass
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
+++ b/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801C5B63-F604-EA45-87E6-A98273F17BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F10B09-3471-D64D-B902-CE6E526BC0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21160" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21160" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="15.2.1" sheetId="1" r:id="rId1"/>
@@ -94,27 +94,6 @@
     <t>Feed Type j </t>
   </si>
   <si>
-    <t>Meat Meal </t>
-  </si>
-  <si>
-    <t>Blood Meal </t>
-  </si>
-  <si>
-    <t>Millrun </t>
-  </si>
-  <si>
-    <t>Whole Sardines </t>
-  </si>
-  <si>
-    <t>Squid </t>
-  </si>
-  <si>
-    <t>Custom Bait </t>
-  </si>
-  <si>
-    <t>Whole Fish </t>
-  </si>
-  <si>
     <t>tonnes</t>
   </si>
   <si>
@@ -125,6 +104,27 @@
   </si>
   <si>
     <t>Low Animal Protein Formulated Feed</t>
+  </si>
+  <si>
+    <t>Meat Meal</t>
+  </si>
+  <si>
+    <t>Blood Meal</t>
+  </si>
+  <si>
+    <t>Millrun</t>
+  </si>
+  <si>
+    <t>Whole Sardines</t>
+  </si>
+  <si>
+    <t>Squid</t>
+  </si>
+  <si>
+    <t>Whole Fish</t>
+  </si>
+  <si>
+    <t>Custom Bait</t>
   </si>
 </sst>
 </file>
@@ -184,12 +184,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,10 +560,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -589,13 +588,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B11">
         <v>100</v>
       </c>
       <c r="C11">
-        <f>_xlfn.XLOOKUP(A11, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" ref="C11:C18" si="0">_xlfn.XLOOKUP(A11, $G$11:$G$18, $H$11:$H$18)</f>
         <v>0.38600000000000001</v>
       </c>
       <c r="D11">
@@ -603,7 +602,7 @@
         <v>38.6</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H11" s="3">
         <v>0.38600000000000001</v>
@@ -611,21 +610,21 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B12">
         <v>200</v>
       </c>
       <c r="C12">
-        <f>_xlfn.XLOOKUP(A12, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>1.9</v>
       </c>
       <c r="D12">
-        <f t="shared" ref="D12:D18" si="0">B12*C12</f>
+        <f t="shared" ref="D12:D18" si="1">B12*C12</f>
         <v>380</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H12" s="3">
         <v>1.9</v>
@@ -633,21 +632,21 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>300</v>
       </c>
       <c r="C13">
-        <f>_xlfn.XLOOKUP(A13, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H13" s="3">
         <v>0.3</v>
@@ -655,21 +654,21 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B14">
         <v>400</v>
       </c>
       <c r="C14">
-        <f>_xlfn.XLOOKUP(A14, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H14" s="3">
         <v>0.3</v>
@@ -677,43 +676,43 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>500</v>
       </c>
       <c r="C15">
-        <f>_xlfn.XLOOKUP(A15, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>2.2000000000000002</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1100</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" s="4">
+        <v>13</v>
+      </c>
+      <c r="H15" s="3">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>600</v>
       </c>
       <c r="C16">
-        <f>_xlfn.XLOOKUP(A16, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>180</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H16" s="3">
         <v>0.3</v>
@@ -721,21 +720,21 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>700</v>
       </c>
       <c r="C17">
-        <f>_xlfn.XLOOKUP(A17, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>210</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H17" s="3">
         <v>0.3</v>
@@ -743,21 +742,21 @@
     </row>
     <row r="18" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>800</v>
       </c>
       <c r="C18">
-        <f>_xlfn.XLOOKUP(A18, $G$11:$G$18, $H$11:$H$18)</f>
+        <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H18" s="3">
         <v>0.08</v>
@@ -765,7 +764,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
test(calculators): added test cases for every possible feed type at present
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
+++ b/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F10B09-3471-D64D-B902-CE6E526BC0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756F7828-56A6-4A49-8EC7-FF1B941F8C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21160" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="840" yWindow="1580" windowWidth="25020" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="15.2.1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="56">
   <si>
     <t>input</t>
   </si>
@@ -126,12 +126,117 @@
   <si>
     <t>Custom Bait</t>
   </si>
+  <si>
+    <t>Region (j)</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Barley grain</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>NSW</t>
+  </si>
+  <si>
+    <t>NT</t>
+  </si>
+  <si>
+    <t>QLD</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>TAS</t>
+  </si>
+  <si>
+    <t>VIC</t>
+  </si>
+  <si>
+    <t>WA</t>
+  </si>
+  <si>
+    <t>Maize grain</t>
+  </si>
+  <si>
+    <t>Sorghum grain</t>
+  </si>
+  <si>
+    <t>Wheat grain</t>
+  </si>
+  <si>
+    <t>Cereal hay</t>
+  </si>
+  <si>
+    <t>Cereal silage</t>
+  </si>
+  <si>
+    <t>Lucerne hay</t>
+  </si>
+  <si>
+    <t>Maize silage</t>
+  </si>
+  <si>
+    <t>Oaten hay</t>
+  </si>
+  <si>
+    <t>Pasture hay</t>
+  </si>
+  <si>
+    <t>Wheat bran</t>
+  </si>
+  <si>
+    <t>Canola meal</t>
+  </si>
+  <si>
+    <t>Soybean meal</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Feed for chickens</t>
+  </si>
+  <si>
+    <t>Feed for pigs</t>
+  </si>
+  <si>
+    <t>Feed for dairy calves</t>
+  </si>
+  <si>
+    <t>Feed for dairy cows</t>
+  </si>
+  <si>
+    <t>Lick block, dry season mix</t>
+  </si>
+  <si>
+    <t>Lick block, weaner</t>
+  </si>
+  <si>
+    <t>Canola oil</t>
+  </si>
+  <si>
+    <t>Cotton seed</t>
+  </si>
+  <si>
+    <t>Lick block, mineral</t>
+  </si>
+  <si>
+    <t>Bentonite</t>
+  </si>
+  <si>
+    <t>Molasses</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -157,8 +262,14 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -168,6 +279,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -184,11 +307,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,299 +650,2393 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A5:H26"/>
+  <dimension ref="A5:I100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="D5" s="2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C7">
         <v>257</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>258</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>256</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
         <v>0</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>1</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B11">
-        <v>100</v>
-      </c>
       <c r="C11">
-        <f t="shared" ref="C11:C18" si="0">_xlfn.XLOOKUP(A11, $G$11:$G$18, $H$11:$H$18)</f>
+        <v>100</v>
+      </c>
+      <c r="D11">
+        <f>I11</f>
         <v>0.38600000000000001</v>
       </c>
-      <c r="D11">
-        <f>B11*C11</f>
+      <c r="E11">
+        <f>C11*D11</f>
         <v>38.6</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="5"/>
+      <c r="I11" s="5">
         <v>0.38600000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>200</v>
       </c>
-      <c r="C12">
-        <f t="shared" si="0"/>
+      <c r="D12">
+        <f t="shared" ref="D12:D75" si="0">I12</f>
         <v>1.9</v>
       </c>
-      <c r="D12">
-        <f t="shared" ref="D12:D18" si="1">B12*C12</f>
+      <c r="E12">
+        <f t="shared" ref="E12:E75" si="1">C12*D12</f>
         <v>380</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="5"/>
+      <c r="I12" s="5">
         <v>1.9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>300</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="5"/>
+      <c r="I13" s="5">
         <v>0.3</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>400</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="5"/>
+      <c r="I14" s="5">
         <v>0.3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
+      <c r="C15">
         <v>500</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <f t="shared" si="0"/>
         <v>2.2000000000000002</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <f t="shared" si="1"/>
         <v>1100</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="5"/>
+      <c r="I15" s="5">
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B16">
+      <c r="C16">
         <v>600</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <f t="shared" si="1"/>
         <v>180</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="5"/>
+      <c r="I16" s="5">
         <v>0.3</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17">
+      <c r="C17">
         <v>700</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <f t="shared" si="1"/>
         <v>210</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="5"/>
+      <c r="I17" s="5">
         <v>0.3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B18">
+      <c r="C18">
         <v>800</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <f t="shared" si="1"/>
         <v>64</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="5"/>
+      <c r="I18" s="5">
         <v>0.08</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19">
+        <v>100</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>23.9</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="6">
+        <v>0.23899999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20">
+        <v>100</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>25.6</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="7">
+        <v>0.25600000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21">
+        <v>100</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>0.33200000000000002</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>33.200000000000003</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21" s="7">
+        <v>0.33200000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22">
+        <v>100</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>0.26900000000000002</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>26.900000000000002</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="7">
+        <v>0.26900000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23">
+        <v>100</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>0.223</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>22.3</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23" s="7">
+        <v>0.223</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24">
+        <v>100</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>0.307</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>30.7</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" s="7">
+        <v>0.307</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25">
+        <v>100</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="1"/>
+        <v>24.099999999999998</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25" s="7">
+        <v>0.24099999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26">
+        <v>100</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="1"/>
+        <v>23.599999999999998</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I26" s="7">
+        <v>0.23599999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27">
+        <v>100</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="0"/>
+        <v>0.18099999999999999</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="1"/>
+        <v>18.099999999999998</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="7">
+        <v>0.18099999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28">
+        <v>100</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="0"/>
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="1"/>
+        <v>16.900000000000002</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="7">
+        <v>0.16900000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29">
+        <v>100</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="0"/>
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="1"/>
+        <v>25.6</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I29" s="7">
+        <v>0.25600000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>100</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="0"/>
+        <v>0.186</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="1"/>
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I30" s="7">
+        <v>0.186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31">
+        <v>100</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="0"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="1"/>
+        <v>17.599999999999998</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I31" s="7">
+        <v>0.17599999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32">
+        <v>100</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="0"/>
+        <v>0.159</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="1"/>
+        <v>15.9</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I32" s="7">
+        <v>0.159</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33">
+        <v>100</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="1"/>
+        <v>28.499999999999996</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I33" s="7">
+        <v>0.28499999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34">
+        <v>100</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>0.23200000000000001</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="1"/>
+        <v>23.200000000000003</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I34" s="7">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35">
+        <v>100</v>
+      </c>
+      <c r="D35">
+        <f t="shared" si="0"/>
+        <v>0.23200000000000001</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="1"/>
+        <v>23.200000000000003</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I35" s="7">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36">
+        <v>100</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="0"/>
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="1"/>
+        <v>23.1</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="7">
+        <v>0.23100000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37">
+        <v>100</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="0"/>
+        <v>0.218</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="1"/>
+        <v>21.8</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I37" s="7">
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38">
+        <v>100</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="0"/>
+        <v>0.246</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="1"/>
+        <v>24.6</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I38" s="7">
+        <v>0.246</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39">
+        <v>100</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="0"/>
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="1"/>
+        <v>26.8</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I39" s="7">
+        <v>0.26800000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40">
+        <v>100</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="0"/>
+        <v>0.28199999999999997</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="1"/>
+        <v>28.199999999999996</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I40" s="7">
+        <v>0.28199999999999997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C41">
+        <v>100</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="1"/>
+        <v>38.5</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I41" s="7">
+        <v>0.38500000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
+      </c>
+      <c r="D42">
+        <f>I42</f>
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="1"/>
+        <v>29.599999999999998</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I42" s="7">
+        <v>0.29599999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
+      </c>
+      <c r="D43">
+        <f t="shared" si="0"/>
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="1"/>
+        <v>24.099999999999998</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I43" s="7">
+        <v>0.24099999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44">
+        <v>100</v>
+      </c>
+      <c r="D44">
+        <f t="shared" si="0"/>
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="1"/>
+        <v>33.800000000000004</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I44" s="7">
+        <v>0.33800000000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C45">
+        <v>100</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="0"/>
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="1"/>
+        <v>26.6</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I45" s="7">
+        <v>0.26600000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C46">
+        <v>100</v>
+      </c>
+      <c r="D46">
+        <f t="shared" si="0"/>
+        <v>0.26100000000000001</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="1"/>
+        <v>26.1</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I46" s="7">
+        <v>0.26100000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C47">
+        <v>100</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="0"/>
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="1"/>
+        <v>11.700000000000001</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I47" s="7">
+        <v>0.11700000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48">
+        <v>100</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="0"/>
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="1"/>
+        <v>11.600000000000001</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I48" s="7">
+        <v>0.11600000000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49">
+        <v>100</v>
+      </c>
+      <c r="D49">
+        <f t="shared" si="0"/>
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="1"/>
+        <v>11.799999999999999</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I49" s="7">
+        <v>0.11799999999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50">
+        <v>100</v>
+      </c>
+      <c r="D50">
+        <f t="shared" si="0"/>
+        <v>0.111</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="1"/>
+        <v>11.1</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I50" s="7">
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C51">
+        <v>100</v>
+      </c>
+      <c r="D51">
+        <f t="shared" si="0"/>
+        <v>0.13900000000000001</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="1"/>
+        <v>13.900000000000002</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I51" s="7">
+        <v>0.13900000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52">
+        <v>100</v>
+      </c>
+      <c r="D52">
+        <f t="shared" si="0"/>
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="1"/>
+        <v>11.600000000000001</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I52" s="7">
+        <v>0.11600000000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C53">
+        <v>100</v>
+      </c>
+      <c r="D53">
+        <f t="shared" si="0"/>
+        <v>0.122</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="1"/>
+        <v>12.2</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I53" s="7">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A54" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C54">
+        <v>100</v>
+      </c>
+      <c r="D54">
+        <f t="shared" si="0"/>
+        <v>7.4399999999999994E-2</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="1"/>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H54" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I54" s="7">
+        <v>7.4399999999999994E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A55" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C55">
+        <v>100</v>
+      </c>
+      <c r="D55">
+        <f t="shared" si="0"/>
+        <v>7.4399999999999994E-2</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="1"/>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I55" s="7">
+        <v>7.4399999999999994E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56">
+        <v>100</v>
+      </c>
+      <c r="D56">
+        <f t="shared" si="0"/>
+        <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="1"/>
+        <v>7.9</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I56" s="7">
+        <v>7.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57">
+        <v>100</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="0"/>
+        <v>7.0599999999999996E-2</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="1"/>
+        <v>7.06</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I57" s="7">
+        <v>7.0599999999999996E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C58">
+        <v>100</v>
+      </c>
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>8.0799999999999997E-2</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="1"/>
+        <v>8.08</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I58" s="7">
+        <v>8.0799999999999997E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59">
+        <v>100</v>
+      </c>
+      <c r="D59">
+        <f t="shared" si="0"/>
+        <v>7.3599999999999999E-2</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="1"/>
+        <v>7.3599999999999994</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I59" s="7">
+        <v>7.3599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A60" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C60">
+        <v>100</v>
+      </c>
+      <c r="D60">
+        <f t="shared" si="0"/>
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="1"/>
+        <v>11.700000000000001</v>
+      </c>
+      <c r="G60" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I60" s="7">
+        <v>0.11700000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C61">
+        <v>100</v>
+      </c>
+      <c r="D61">
+        <f t="shared" si="0"/>
+        <v>0.113</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="1"/>
+        <v>11.3</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I61" s="7">
+        <v>0.113</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C62">
+        <v>100</v>
+      </c>
+      <c r="D62">
+        <f t="shared" si="0"/>
+        <v>0.14299999999999999</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="1"/>
+        <v>14.299999999999999</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I62" s="7">
+        <v>0.14299999999999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63">
+        <v>100</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="0"/>
+        <v>0.106</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="1"/>
+        <v>10.6</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H63" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I63" s="7">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64">
+        <v>100</v>
+      </c>
+      <c r="D64">
+        <f t="shared" si="0"/>
+        <v>0.113</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="1"/>
+        <v>11.3</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H64" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I64" s="7">
+        <v>0.113</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C65">
+        <v>100</v>
+      </c>
+      <c r="D65">
+        <f t="shared" si="0"/>
+        <v>0.106</v>
+      </c>
+      <c r="E65">
+        <f t="shared" si="1"/>
+        <v>10.6</v>
+      </c>
+      <c r="G65" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H65" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I65" s="7">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C66">
+        <v>100</v>
+      </c>
+      <c r="D66">
+        <f>I66</f>
+        <v>0.16300000000000001</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="1"/>
+        <v>16.3</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H66" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I66" s="7">
+        <v>0.16300000000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C67">
+        <v>100</v>
+      </c>
+      <c r="D67">
+        <f t="shared" si="0"/>
+        <v>0.12</v>
+      </c>
+      <c r="E67">
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C22" t="s">
+      <c r="G67" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H67" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I67" s="7">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C68">
+        <v>100</v>
+      </c>
+      <c r="D68">
+        <f t="shared" si="0"/>
+        <v>0.11899999999999999</v>
+      </c>
+      <c r="E68">
+        <f t="shared" si="1"/>
+        <v>11.899999999999999</v>
+      </c>
+      <c r="G68" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I68" s="7">
+        <v>0.11899999999999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A69" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C69">
+        <v>100</v>
+      </c>
+      <c r="D69">
+        <f t="shared" si="0"/>
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="1"/>
+        <v>11.700000000000001</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H69" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I69" s="7">
+        <v>0.11700000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A70" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C70">
+        <v>100</v>
+      </c>
+      <c r="D70">
+        <f t="shared" si="0"/>
+        <v>0.114</v>
+      </c>
+      <c r="E70">
+        <f t="shared" si="1"/>
+        <v>11.4</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H70" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I70" s="7">
+        <v>0.114</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A71" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C71">
+        <v>100</v>
+      </c>
+      <c r="D71">
+        <f t="shared" si="0"/>
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="E71">
+        <f t="shared" si="1"/>
+        <v>11.799999999999999</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I71" s="7">
+        <v>0.11799999999999999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A72" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C72">
+        <v>100</v>
+      </c>
+      <c r="D72">
+        <f t="shared" si="0"/>
+        <v>0.124</v>
+      </c>
+      <c r="E72">
+        <f t="shared" si="1"/>
+        <v>12.4</v>
+      </c>
+      <c r="G72" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H72" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I72" s="7">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C73">
+        <v>100</v>
+      </c>
+      <c r="D73">
+        <f t="shared" si="0"/>
+        <v>0.33900000000000002</v>
+      </c>
+      <c r="E73">
+        <f t="shared" si="1"/>
+        <v>33.900000000000006</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I73" s="7">
+        <v>0.33900000000000002</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A74" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C74">
+        <v>100</v>
+      </c>
+      <c r="D74">
+        <f t="shared" si="0"/>
+        <v>0.311</v>
+      </c>
+      <c r="E74">
+        <f t="shared" si="1"/>
+        <v>31.1</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H74" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I74" s="7">
+        <v>0.311</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A75" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C75">
+        <v>100</v>
+      </c>
+      <c r="D75">
+        <f t="shared" si="0"/>
+        <v>0.254</v>
+      </c>
+      <c r="E75">
+        <f t="shared" si="1"/>
+        <v>25.4</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I75" s="7">
+        <v>0.254</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A76" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76">
+        <v>100</v>
+      </c>
+      <c r="D76">
+        <f t="shared" ref="D76:D93" si="2">I76</f>
+        <v>0.313</v>
+      </c>
+      <c r="E76">
+        <f t="shared" ref="E76:E93" si="3">C76*D76</f>
+        <v>31.3</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H76" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I76" s="7">
+        <v>0.313</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C77">
+        <v>100</v>
+      </c>
+      <c r="D77">
+        <f t="shared" si="2"/>
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="E77">
+        <f t="shared" si="3"/>
+        <v>39.800000000000004</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I77" s="7">
+        <v>0.39800000000000002</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A78" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C78">
+        <v>100</v>
+      </c>
+      <c r="D78">
+        <f t="shared" si="2"/>
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="E78">
+        <f t="shared" si="3"/>
+        <v>34.5</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H78" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I78" s="7">
+        <v>0.34499999999999997</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A79" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C79">
+        <v>100</v>
+      </c>
+      <c r="D79">
+        <f t="shared" si="2"/>
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="E79">
+        <f t="shared" si="3"/>
+        <v>36.799999999999997</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I79" s="7">
+        <v>0.36799999999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A80" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C80">
+        <v>100</v>
+      </c>
+      <c r="D80">
+        <f t="shared" si="2"/>
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="E80">
+        <f t="shared" si="3"/>
+        <v>19.600000000000001</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H80" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I80" s="7">
+        <v>0.19600000000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A81" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C81">
+        <v>100</v>
+      </c>
+      <c r="D81">
+        <f t="shared" si="2"/>
+        <v>0.24399999999999999</v>
+      </c>
+      <c r="E81">
+        <f t="shared" si="3"/>
+        <v>24.4</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I81" s="7">
+        <v>0.24399999999999999</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A82" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C82">
+        <v>100</v>
+      </c>
+      <c r="D82">
+        <f t="shared" si="2"/>
+        <v>1.23</v>
+      </c>
+      <c r="E82">
+        <f t="shared" si="3"/>
+        <v>123</v>
+      </c>
+      <c r="G82" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H82" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I82" s="7">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A83" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C83">
+        <v>100</v>
+      </c>
+      <c r="D83">
+        <f t="shared" si="2"/>
+        <v>0.59399999999999997</v>
+      </c>
+      <c r="E83">
+        <f t="shared" si="3"/>
+        <v>59.4</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H83" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I83" s="7">
+        <v>0.59399999999999997</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A84" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C84">
+        <v>100</v>
+      </c>
+      <c r="D84">
+        <f t="shared" si="2"/>
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="E84">
+        <f t="shared" si="3"/>
+        <v>40.300000000000004</v>
+      </c>
+      <c r="G84" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H84" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I84" s="7">
+        <v>0.40300000000000002</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A85" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C85">
+        <v>100</v>
+      </c>
+      <c r="D85">
+        <f t="shared" si="2"/>
+        <v>0.41899999999999998</v>
+      </c>
+      <c r="E85">
+        <f t="shared" si="3"/>
+        <v>41.9</v>
+      </c>
+      <c r="G85" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I85" s="7">
+        <v>0.41899999999999998</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A86" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C86">
+        <v>100</v>
+      </c>
+      <c r="D86">
+        <f t="shared" si="2"/>
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="E86">
+        <f t="shared" si="3"/>
+        <v>33.300000000000004</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H86" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I86" s="7">
+        <v>0.33300000000000002</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>49</v>
+      </c>
+      <c r="C87">
+        <v>100</v>
+      </c>
+      <c r="D87">
+        <f t="shared" si="2"/>
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="E87">
+        <f t="shared" si="3"/>
+        <v>88.1</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H87" s="6"/>
+      <c r="I87" s="6">
+        <v>0.88100000000000001</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>50</v>
+      </c>
+      <c r="C88">
+        <v>100</v>
+      </c>
+      <c r="D88">
+        <f t="shared" si="2"/>
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="E88">
+        <f t="shared" si="3"/>
+        <v>23.1</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H88" s="6"/>
+      <c r="I88" s="6">
+        <v>0.23100000000000001</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>51</v>
+      </c>
+      <c r="B89" t="s">
+        <v>24</v>
+      </c>
+      <c r="C89">
+        <v>100</v>
+      </c>
+      <c r="D89">
+        <f t="shared" si="2"/>
+        <v>0.87</v>
+      </c>
+      <c r="E89">
+        <f t="shared" si="3"/>
+        <v>87</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I89" s="6">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>52</v>
+      </c>
+      <c r="B90" t="s">
+        <v>24</v>
+      </c>
+      <c r="C90">
+        <v>100</v>
+      </c>
+      <c r="D90">
+        <f t="shared" si="2"/>
+        <v>0.19700000000000001</v>
+      </c>
+      <c r="E90">
+        <f t="shared" si="3"/>
+        <v>19.7</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I90" s="6">
+        <v>0.19700000000000001</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>53</v>
+      </c>
+      <c r="C91">
+        <v>100</v>
+      </c>
+      <c r="D91">
+        <f t="shared" si="2"/>
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="E91">
+        <f t="shared" si="3"/>
+        <v>67.7</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H91" s="6"/>
+      <c r="I91" s="6">
+        <v>0.67700000000000005</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>54</v>
+      </c>
+      <c r="C92">
+        <v>100</v>
+      </c>
+      <c r="D92">
+        <f t="shared" si="2"/>
+        <v>6.5199999999999994E-2</v>
+      </c>
+      <c r="E92">
+        <f t="shared" si="3"/>
+        <v>6.52</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H92" s="6"/>
+      <c r="I92" s="6">
+        <v>6.5199999999999994E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>55</v>
+      </c>
+      <c r="B93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C93">
+        <v>100</v>
+      </c>
+      <c r="D93">
+        <f t="shared" si="2"/>
+        <v>0.184</v>
+      </c>
+      <c r="E93">
+        <f t="shared" si="3"/>
+        <v>18.399999999999999</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I93" s="6">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A95" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D96" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B23" s="1" t="s">
+    <row r="97" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C97" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D97" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E97" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B24">
-        <v>100</v>
-      </c>
-      <c r="C24">
+    <row r="98" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C98">
+        <v>100</v>
+      </c>
+      <c r="D98">
         <v>0</v>
       </c>
-      <c r="D24">
-        <f>B24*C24</f>
+      <c r="E98">
+        <f>C98*D98</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B25">
+    <row r="99" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C99">
         <v>200</v>
       </c>
-      <c r="C25">
+      <c r="D99">
         <v>0.1</v>
       </c>
-      <c r="D25">
-        <f>B25*C25</f>
+      <c r="E99">
+        <f>C99*D99</f>
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B26">
+    <row r="100" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C100">
         <v>300</v>
       </c>
-      <c r="C26">
+      <c r="D100">
         <v>0.99</v>
       </c>
-      <c r="D26">
-        <f>B26*C26</f>
+      <c r="E100">
+        <f>C100*D100</f>
         <v>297</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(calculators): draft implementation of module 15.3
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
+++ b/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756F7828-56A6-4A49-8EC7-FF1B941F8C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D84356-6055-D449-AE38-2FED63AD1F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="1580" windowWidth="25020" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1820" yWindow="1500" windowWidth="25020" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="15.2.1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="53">
   <si>
     <t>input</t>
   </si>
@@ -211,19 +211,10 @@
     <t>Feed for dairy cows</t>
   </si>
   <si>
-    <t>Lick block, dry season mix</t>
-  </si>
-  <si>
-    <t>Lick block, weaner</t>
-  </si>
-  <si>
     <t>Canola oil</t>
   </si>
   <si>
     <t>Cotton seed</t>
-  </si>
-  <si>
-    <t>Lick block, mineral</t>
   </si>
   <si>
     <t>Bentonite</t>
@@ -650,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A5:I100"/>
+  <dimension ref="A5:I97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -2510,11 +2501,11 @@
         <v>100</v>
       </c>
       <c r="D76">
-        <f t="shared" ref="D76:D93" si="2">I76</f>
+        <f t="shared" ref="D76:D90" si="2">I76</f>
         <v>0.313</v>
       </c>
       <c r="E76">
-        <f t="shared" ref="E76:E93" si="3">C76*D76</f>
+        <f t="shared" ref="E76:E90" si="3">C76*D76</f>
         <v>31.3</v>
       </c>
       <c r="G76" s="7" t="s">
@@ -2811,74 +2802,79 @@
       <c r="A87" t="s">
         <v>49</v>
       </c>
+      <c r="B87" t="s">
+        <v>24</v>
+      </c>
       <c r="C87">
         <v>100</v>
       </c>
       <c r="D87">
         <f t="shared" si="2"/>
-        <v>0.88100000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="E87">
         <f t="shared" si="3"/>
-        <v>88.1</v>
+        <v>87</v>
       </c>
       <c r="G87" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H87" s="6"/>
+      <c r="H87" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="I87" s="6">
-        <v>0.88100000000000001</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>50</v>
       </c>
+      <c r="B88" t="s">
+        <v>24</v>
+      </c>
       <c r="C88">
         <v>100</v>
       </c>
       <c r="D88">
         <f t="shared" si="2"/>
-        <v>0.23100000000000001</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="E88">
         <f t="shared" si="3"/>
-        <v>23.1</v>
+        <v>19.7</v>
       </c>
       <c r="G88" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H88" s="6"/>
+      <c r="H88" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="I88" s="6">
-        <v>0.23100000000000001</v>
+        <v>0.19700000000000001</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>51</v>
       </c>
-      <c r="B89" t="s">
-        <v>24</v>
-      </c>
       <c r="C89">
         <v>100</v>
       </c>
       <c r="D89">
         <f t="shared" si="2"/>
-        <v>0.87</v>
+        <v>6.5199999999999994E-2</v>
       </c>
       <c r="E89">
         <f t="shared" si="3"/>
-        <v>87</v>
+        <v>6.52</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H89" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="H89" s="6"/>
       <c r="I89" s="6">
-        <v>0.87</v>
+        <v>6.5199999999999994E-2</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
@@ -2886,157 +2882,83 @@
         <v>52</v>
       </c>
       <c r="B90" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C90">
         <v>100</v>
       </c>
       <c r="D90">
         <f t="shared" si="2"/>
-        <v>0.19700000000000001</v>
+        <v>0.184</v>
       </c>
       <c r="E90">
         <f t="shared" si="3"/>
-        <v>19.7</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>52</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I90" s="6">
-        <v>0.19700000000000001</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>53</v>
-      </c>
-      <c r="C91">
-        <v>100</v>
-      </c>
-      <c r="D91">
-        <f t="shared" si="2"/>
-        <v>0.67700000000000005</v>
-      </c>
-      <c r="E91">
-        <f t="shared" si="3"/>
-        <v>67.7</v>
-      </c>
-      <c r="G91" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H91" s="6"/>
-      <c r="I91" s="6">
-        <v>0.67700000000000005</v>
+        <v>0.184</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>54</v>
-      </c>
-      <c r="C92">
-        <v>100</v>
-      </c>
-      <c r="D92">
-        <f t="shared" si="2"/>
-        <v>6.5199999999999994E-2</v>
-      </c>
-      <c r="E92">
-        <f t="shared" si="3"/>
-        <v>6.52</v>
-      </c>
-      <c r="G92" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="H92" s="6"/>
-      <c r="I92" s="6">
-        <v>6.5199999999999994E-2</v>
+      <c r="A92" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>55</v>
-      </c>
-      <c r="B93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C93">
-        <v>100</v>
-      </c>
-      <c r="D93">
-        <f t="shared" si="2"/>
-        <v>0.184</v>
-      </c>
-      <c r="E93">
-        <f t="shared" si="3"/>
-        <v>18.399999999999999</v>
-      </c>
-      <c r="G93" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H93" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="I93" s="6">
-        <v>0.184</v>
+      <c r="D93" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C94" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A95" s="3" t="s">
-        <v>12</v>
+      <c r="C95">
+        <v>100</v>
+      </c>
+      <c r="D95">
+        <v>0</v>
+      </c>
+      <c r="E95">
+        <f>C95*D95</f>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D96" t="s">
-        <v>0</v>
+      <c r="C96">
+        <v>200</v>
+      </c>
+      <c r="D96">
+        <v>0.1</v>
+      </c>
+      <c r="E96">
+        <f>C96*D96</f>
+        <v>20</v>
       </c>
     </row>
     <row r="97" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C97" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="98" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C98">
-        <v>100</v>
-      </c>
-      <c r="D98">
-        <v>0</v>
-      </c>
-      <c r="E98">
-        <f>C98*D98</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C99">
-        <v>200</v>
-      </c>
-      <c r="D99">
-        <v>0.1</v>
-      </c>
-      <c r="E99">
-        <f>C99*D99</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="100" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C100">
+      <c r="C97">
         <v>300</v>
       </c>
-      <c r="D100">
+      <c r="D97">
         <v>0.99</v>
       </c>
-      <c r="E100">
-        <f>C100*D100</f>
+      <c r="E97">
+        <f>C97*D97</f>
         <v>297</v>
       </c>
     </row>

</xml_diff>